<commit_message>
feat: update FIXED excel template with latest WK36 SLA data
</commit_message>
<xml_diff>
--- a/Dashboard_Template_30_Slides_Final_FIXED.xlsx
+++ b/Dashboard_Template_30_Slides_Final_FIXED.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\0_Agent\0_Dashboad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{417FDEE7-6B5D-4AF2-9677-BDA5F5EBC4B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B29AF58-7E43-4A1C-AB5F-089E364B9FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="797" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="797" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Part 1 - Overview" sheetId="1" r:id="rId1"/>
@@ -146,7 +146,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7484" uniqueCount="1661">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7601" uniqueCount="1661">
   <si>
     <t>Slide No</t>
   </si>
@@ -6119,7 +6119,7 @@
         <v>92</v>
       </c>
       <c r="D2">
-        <v>5148057.4000000004</v>
+        <v>5277631.4000000004</v>
       </c>
       <c r="E2" t="s">
         <v>93</v>
@@ -6170,7 +6170,7 @@
         <v>100</v>
       </c>
       <c r="D5">
-        <v>2691184.8400000017</v>
+        <v>2820758.8400000017</v>
       </c>
       <c r="E5" t="s">
         <v>101</v>
@@ -6288,6 +6288,9 @@
       <c r="C12" t="s">
         <v>115</v>
       </c>
+      <c r="D12">
+        <v>346396.40000000031</v>
+      </c>
       <c r="E12" t="s">
         <v>116</v>
       </c>
@@ -6303,7 +6306,7 @@
         <v>118</v>
       </c>
       <c r="D13">
-        <v>5779708.3399999999</v>
+        <v>6126104.7400000002</v>
       </c>
       <c r="E13" t="s">
         <v>119</v>
@@ -6320,7 +6323,7 @@
         <v>120</v>
       </c>
       <c r="D14">
-        <v>6985932.2116510943</v>
+        <v>6982082.2116510943</v>
       </c>
       <c r="E14" t="s">
         <v>121</v>
@@ -6558,7 +6561,7 @@
         <v>135</v>
       </c>
       <c r="D28">
-        <v>427765</v>
+        <v>501518</v>
       </c>
       <c r="E28" t="s">
         <v>136</v>
@@ -6604,7 +6607,7 @@
         <v>141</v>
       </c>
       <c r="D30">
-        <v>5107</v>
+        <v>10214</v>
       </c>
       <c r="E30" t="s">
         <v>136</v>
@@ -6627,7 +6630,7 @@
         <v>143</v>
       </c>
       <c r="D31">
-        <v>4489699</v>
+        <v>4540413</v>
       </c>
       <c r="E31" t="s">
         <v>136</v>
@@ -6840,7 +6843,7 @@
         <v>164</v>
       </c>
       <c r="D43">
-        <v>1486806.8499999996</v>
+        <v>1833203.25</v>
       </c>
       <c r="E43" t="s">
         <v>164</v>
@@ -7380,7 +7383,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:BP328"/>
+  <dimension ref="A1:BP445"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:68" x14ac:dyDescent="0.25">
@@ -64442,6 +64445,591 @@
     </row>
     <row r="328" spans="1:68" x14ac:dyDescent="0.25">
       <c r="BP328" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="329" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="BP329" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="330" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="BP330" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="331" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="BP331" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="332" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="BP332" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="333" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="BP333" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="334" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="BP334" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="335" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="BP335" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="336" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="BP336" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="337" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP337" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="338" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP338" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="339" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP339" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="340" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP340" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="341" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP341" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="342" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP342" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="343" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP343" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="344" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP344" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="345" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP345" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="346" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP346" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="347" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP347" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="348" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP348" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="349" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP349" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="350" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP350" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="351" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP351" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="352" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP352" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="353" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP353" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="354" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP354" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="355" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP355" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="356" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP356" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="357" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP357" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="358" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP358" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="359" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP359" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="360" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP360" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="361" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP361" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="362" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP362" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="363" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP363" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="364" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP364" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="365" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP365" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="366" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP366" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="367" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP367" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="368" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP368" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="369" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP369" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="370" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP370" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="371" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP371" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="372" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP372" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="373" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP373" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="374" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP374" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="375" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP375" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="376" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP376" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="377" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP377" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="378" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP378" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="379" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP379" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="380" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP380" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="381" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP381" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="382" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP382" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="383" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP383" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="384" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP384" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="385" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP385" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="386" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP386" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="387" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP387" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="388" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP388" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="389" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP389" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="390" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP390" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="391" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP391" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="392" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP392" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="393" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP393" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="394" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP394" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="395" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP395" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="396" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP396" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="397" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP397" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="398" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP398" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="399" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP399" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="400" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP400" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="401" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP401" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="402" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP402" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="403" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP403" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="404" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP404" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="405" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP405" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="406" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP406" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="407" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP407" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="408" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP408" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="409" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP409" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="410" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP410" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="411" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP411" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="412" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP412" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="413" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP413" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="414" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP414" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="415" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP415" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="416" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP416" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="417" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP417" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="418" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP418" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="419" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP419" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="420" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP420" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="421" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP421" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="422" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP422" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="423" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP423" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="424" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP424" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="425" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP425" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="426" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP426" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="427" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP427" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="428" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP428" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="429" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP429" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="430" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP430" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="431" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP431" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="432" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP432" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="433" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP433" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="434" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP434" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="435" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP435" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="436" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP436" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="437" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP437" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="438" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP438" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="439" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP439" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="440" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP440" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="441" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP441" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="442" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP442" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="443" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP443" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="444" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP444" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="445" spans="68:68" x14ac:dyDescent="0.25">
+      <c r="BP445" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>